<commit_message>
feat(analytics): add venue analytics
</commit_message>
<xml_diff>
--- a/project_tracker.xlsx
+++ b/project_tracker.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -794,12 +794,24 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Player batting/bowling, team batting/bowling, match summary/innings, and venue analytics implemented and verified against PostgreSQL.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1542,6 +1554,80 @@
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Added branch/commit/PR workflow guidance for solo development simulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Implement match analytics</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Match summary and innings analytics implemented; verified across multiple real matches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Implement venue analytics</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Venue statistics and top-venues analytics implemented; 9 venue tests and real PostgreSQL validation passed.</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2009,6 +2095,28 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Do not silently canonicalize venue-name variants in analytics</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Venue aliases can represent the same physical venue; merging them inside analytics without an explicit master-data rule could change historical aggregates and make the transformation non-auditable.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: document team head-to-head analytics
</commit_message>
<xml_diff>
--- a/project_tracker.xlsx
+++ b/project_tracker.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Tasks" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,27 +12,24 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture Decisions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tasks'!$A$1:$G$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Project Tasks'!$A$1:$G$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Architecture Decisions'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Architecture Decisions'!$A$1:$D$16</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -54,21 +52,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -431,1127 +419,1167 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="6"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Project structure</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Initial repository structure created</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Setup</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Conda environment</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>IPL_Intelligence_Platform / Python 3.12.13</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Cricsheet dataset profiling</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Profiled raw JSON dataset</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Database</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>PostgreSQL verification</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>PostgreSQL 17.6 service verified</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>005</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Database</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Python database connection</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>SQLAlchemy connection test successful</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>006</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Database</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Database schema design</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Finalized PostgreSQL dim/fact model plus ETL audit and DQ issue tables.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>007</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>JSON ingestion pipeline</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>End-to-end JSON ingestion completed; 1,243/1,243 files successful.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>008</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Validation and data-quality checks</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Structural validation + DQ framework implemented; 60 warnings, 0 blocking errors in full run.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>009</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Player/team/venue analytics</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Player batting/bowling, team batting/bowling, match summary/innings, and venue analytics implemented and verified against PostgreSQL.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>010</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>ML</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Win prediction feature engineering</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>011</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>ML</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Model training and evaluation</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>012</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>GenAI</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>GenAI assistant</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>013</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>RAG</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>RAG knowledge pipeline</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>014</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>API</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Backend API</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>User interface</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>016</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Production deployment</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Inspect Cricsheet source schema</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>46260</v>
-      </c>
-      <c r="G18" s="3" t="n"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Build JSON reader</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="4" t="n">
-        <v>46260</v>
-      </c>
-      <c r="G19" s="3" t="n"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Build match parser</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="4" t="n">
-        <v>46260</v>
-      </c>
-      <c r="G20" s="3" t="n"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Build match validator</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Structural match validator implemented and negative cases verified.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Build transformation layer</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Validated domain records transformed into database-ready package.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Build PostgreSQL loader</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Loaded dimensions, match relationships, innings, deliveries, extras and wickets.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Implement ETL audit logging</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>ETL run and file-level audit status/stage/duration/error tracking implemented.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Full IPL ingestion run</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Run 7: 1,243 discovered, 1,243 processed, 1,243 successful, 0 failed.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Verify loader idempotency</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Reran match 1082591; business-row counts unchanged.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Source integrity verification</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>1,243 JSON files; numeric/unique match IDs; no duplicate IDs.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>ETL</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Source-to-database reconciliation</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Matches, innings, deliveries, extras and wickets all reconciled exactly.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Data-quality rule framework</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Severity-based DQ result model with ERROR/WARNING handling implemented.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Persist data-quality issues</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Persisted file-level DQ issues into etl_file_quality_issue and verified audit relationship.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Full DQ warning analysis</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Full dataset: DQ010=51 warnings, DQ011=9 warnings, total=60, errors=0.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Full regression test suite</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>23 tests passed after DQ integration.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Update engineering documentation</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Updated architecture, data dictionary, database, ETL, testing, troubleshooting, DQ and change log docs.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Project Management</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Professional Git workflow</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Abhay</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Added branch/commit/PR workflow guidance for solo development simulation.</t>
         </is>
@@ -1627,12 +1655,49 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Venue statistics and top-venues analytics implemented; 9 venue tests and real PostgreSQL validation passed.</t>
+          <t>Venue statistics and top-venues analytics; 9 venue tests and real PostgreSQL validation passed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Team head-to-head analytics</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Abhay</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Outcome preservation/backfill, overall H2H, season-wise H2H, 10 unit tests, PostgreSQL integration verification; full regression 64 passed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G34"/>
+  <autoFilter ref="A1:G37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1644,145 +1709,145 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Issue ID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cause</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Solution</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>BUG-001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Conda not recognized in PowerShell</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Shell integration / execution policy</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Configure PowerShell for Conda and verify activation</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>BUG-002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>No module named 'src'</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Script executed directly from scripts directory context</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Run as module: python -m scripts.test_database_connection</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>BUG-003</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>pip path appeared to use user-level Python</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>User-level pip was visible during initial diagnostic</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Verified environment pip/package import paths using conda list, where.exe, sys.path and pip.__file__</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>BUG-004</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Simple over_number + ball_number uniqueness falsely flagged valid illegal deliveries</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Source delivery numbering is not a safe uniqueness key around wides/no-balls</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Use delivery_sequence and enforce uniqueness on innings_id + over_number + delivery_sequence</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -1800,296 +1865,296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Use PostgreSQL</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Reliable relational database for detailed cricket event data and analytics</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Use SQLAlchemy</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Centralize database connectivity and support maintainable Python database code</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Preserve raw JSON</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Maintain reproducibility and data lineage</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Use delivery-level fact data</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Preserve detailed event-level information for analytics and ML feature generation</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Separate structured data from RAG knowledge</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Avoid using vector search where relational/analytical queries are more appropriate</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Normalize historical team aliases</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Prevent renamed IPL franchises from becoming separate analytical teams</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Use delivery_sequence for delivery-position uniqueness</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Avoid false duplicate detection caused by illegal deliveries and source ball numbering</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>Separate DQ issues into an audit table</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Keep data-quality observations queryable without mixing them into cricket fact tables</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Treat DQ warnings as non-blocking</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Incomplete but usable records can load while remaining visible for audit</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Treat DQ errors as blocking</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Prevent structurally/logically invalid records from reaching analytical tables</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Require source-to-DB reconciliation before downstream analytics</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Establish a measurable data-integrity gate before ML/analytics</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Use logical Git commits and PRs</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Simulate professional team development workflow and maintain reviewable history</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
@@ -2117,8 +2182,52 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Preserve match outcome_result and outcome_deciding_team_id separately from winner_id</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Preserve source tie/no-result semantics and retain Super Over/eliminator deciding-team information without converting ties into ordinary wins.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Perform H2H aggregation in PostgreSQL using match_team pair joins</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Identify matches where both teams participated and aggregate close to the data source rather than loading match history into Python.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>